<commit_message>
Daily run 2026-10-20: ai-chatbot-cost post, SEO meta set in generator, FB #3, Tuesday draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPVrWiXaNrFkjT3XxN8ywn
</commit_message>
<xml_diff>
--- a/checklist/Blog content checklist.xlsx
+++ b/checklist/Blog content checklist.xlsx
@@ -709,12 +709,18 @@
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="n"/>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/ai-chatbot-cost</t>
+        </is>
+      </c>
       <c r="J6" s="18" t="n"/>
-      <c r="K6" s="20" t="n"/>
+      <c r="K6" s="19" t="n">
+        <v>46315</v>
+      </c>
       <c r="L6" s="18" t="n"/>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="13">
@@ -1090,6 +1096,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Publish ai-chatbot-human-handoff; Friday digest 2026-10-23
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPVrWiXaNrFkjT3XxN8ywn
</commit_message>
<xml_diff>
--- a/checklist/Blog content checklist.xlsx
+++ b/checklist/Blog content checklist.xlsx
@@ -895,12 +895,18 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="n"/>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/ai-chatbot-human-handoff</t>
+        </is>
+      </c>
       <c r="J10" s="18" t="n"/>
-      <c r="K10" s="20" t="n"/>
+      <c r="K10" s="19" t="n">
+        <v>46318</v>
+      </c>
       <c r="L10" s="18" t="n"/>
     </row>
     <row r="11" ht="23.25" customHeight="1" s="13">
@@ -1111,6 +1117,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId5"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Publish mcp-ai-agent-business-tools and rag-ai-agent-business-knowledge; listings, queue, sitemap; per-post list padding
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPVrWiXaNrFkjT3XxN8ywn
</commit_message>
<xml_diff>
--- a/checklist/Blog content checklist.xlsx
+++ b/checklist/Blog content checklist.xlsx
@@ -1138,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -1672,33 +1672,88 @@
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I14" s="18" t="n"/>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/mcp-ai-agent-business-tools</t>
+        </is>
+      </c>
       <c r="J14" s="18" t="n"/>
-      <c r="K14" s="20" t="n"/>
+      <c r="K14" s="19" t="n">
+        <v>46322</v>
+      </c>
       <c r="L14" s="18" t="n"/>
     </row>
-    <row r="16" ht="15" customHeight="1" s="13">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>How to Ground an AI Agent in Your Business Knowledge (RAG Explained for Business Owners)</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Solution-aware</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>RAG for business, AI agent knowledge base</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Shows Dijae's long-standing knowledge-base (RAG) agent work; uses his own Botcake Knowledge screenshots; added by Dijae Oct 27 2026</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="B16" s="22">
-        <f>COUNTIF(H5:H14,"Published")&amp;" of "&amp;COUNTA(C5:C14)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="I15" s="18" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/rag-ai-agent-business-knowledge</t>
+        </is>
+      </c>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="19" t="n">
+        <v>46322</v>
+      </c>
+      <c r="L15" s="18" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="13"/>
     <row r="17" ht="15" customHeight="1" s="13">
       <c r="A17" s="21" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="B17" s="22">
+        <f>COUNTIF(H5:H15,"Published")&amp;" of "&amp;COUNTA(C5:C15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
           <t>Need recording</t>
         </is>
       </c>
-      <c r="B17" s="22">
-        <f>COUNTIF(G5:G14,"Yes*")</f>
+      <c r="B18" s="22">
+        <f>COUNTIF(G5:G15,"Yes*")</f>
         <v/>
       </c>
     </row>
@@ -1710,7 +1765,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H5:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Planned,Recording needed,Drafting,Published"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1721,6 +1776,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" display="https://www.dijaedadula.com/ai-automation-clinics-med-spas" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" display="https://www.dijaedadula.com/price-ai-automation-services" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId7"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Oct 30: AI agent monitoring post (#14), listings, interlinks, Friday digest 1019, FB get-more-clients-with-ai
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPVrWiXaNrFkjT3XxN8ywn
</commit_message>
<xml_diff>
--- a/checklist/Blog content checklist.xlsx
+++ b/checklist/Blog content checklist.xlsx
@@ -1859,12 +1859,18 @@
       </c>
       <c r="H18" s="17" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I18" s="17" t="n"/>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/ai-agent-monitoring-weekly-review</t>
+        </is>
+      </c>
       <c r="J18" s="17" t="n"/>
-      <c r="K18" s="19" t="n"/>
+      <c r="K18" s="22" t="n">
+        <v>46325</v>
+      </c>
       <c r="L18" s="17" t="inlineStr">
         <is>
           <t>Added by Dijae Oct 28 2026</t>
@@ -2330,6 +2336,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" display="https://www.dijaedadula.com/rag-ai-agent-business-knowledge" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" display="https://www.dijaedadula.com/ai-agent-guardrails" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId10"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Oct 31: CRM pipeline stages post (#15), listings, interlinks, FB what-does-an-ai-trainer-do
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPVrWiXaNrFkjT3XxN8ywn
</commit_message>
<xml_diff>
--- a/checklist/Blog content checklist.xlsx
+++ b/checklist/Blog content checklist.xlsx
@@ -1911,12 +1911,18 @@
       </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="n"/>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>https://www.dijaedadula.com/crm-pipeline-stages-service-business</t>
+        </is>
+      </c>
       <c r="J19" s="17" t="n"/>
-      <c r="K19" s="19" t="n"/>
+      <c r="K19" s="22" t="n">
+        <v>46326</v>
+      </c>
       <c r="L19" s="17" t="inlineStr">
         <is>
           <t>Added by Dijae Oct 28 2026</t>
@@ -2337,6 +2343,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" display="https://www.dijaedadula.com/ai-agent-guardrails" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId11"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>